<commit_message>
Add Feb 2026 data
</commit_message>
<xml_diff>
--- a/data/Fatmeter_Data_Feb_2026.xlsx
+++ b/data/Fatmeter_Data_Feb_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sean.rohan\Work\afsc\fatmeter\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79B2B919-D245-43D1-B7D9-32A60092EBE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FAD1B64-35B7-4884-B994-FDBF6BFB9E21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1905" yWindow="1905" windowWidth="38700" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7965" yWindow="2220" windowWidth="38700" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="11" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1616" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1614" uniqueCount="79">
   <si>
     <t>Distell tissue</t>
   </si>
@@ -969,7 +969,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB338"/>
+  <dimension ref="A1:AB342"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" style="1" customWidth="1"/>
@@ -21114,6 +21114,194 @@
         <v>47.1</v>
       </c>
     </row>
+    <row r="339" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A339" s="1">
+        <v>449</v>
+      </c>
+      <c r="B339" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C339" s="1">
+        <v>202301</v>
+      </c>
+      <c r="D339" s="1">
+        <v>162</v>
+      </c>
+      <c r="E339" s="1">
+        <v>138</v>
+      </c>
+      <c r="H339">
+        <v>57.349710000000002</v>
+      </c>
+      <c r="I339">
+        <v>-169.59164999999999</v>
+      </c>
+      <c r="J339" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K339" s="1">
+        <v>4</v>
+      </c>
+      <c r="L339" s="1">
+        <v>65</v>
+      </c>
+      <c r="M339" s="1">
+        <v>2936</v>
+      </c>
+      <c r="N339" s="1">
+        <v>68</v>
+      </c>
+      <c r="O339" s="1">
+        <v>86</v>
+      </c>
+      <c r="P339" s="1">
+        <v>30</v>
+      </c>
+      <c r="T339" s="1">
+        <v>4.7</v>
+      </c>
+      <c r="U339" s="1">
+        <v>51.3</v>
+      </c>
+    </row>
+    <row r="340" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A340" s="1">
+        <v>450</v>
+      </c>
+      <c r="B340" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C340" s="1">
+        <v>202301</v>
+      </c>
+      <c r="D340" s="1">
+        <v>162</v>
+      </c>
+      <c r="E340" s="1">
+        <v>138</v>
+      </c>
+      <c r="H340">
+        <v>57.349710000000002</v>
+      </c>
+      <c r="I340">
+        <v>-169.59164999999999</v>
+      </c>
+      <c r="J340" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K340" s="1">
+        <v>4</v>
+      </c>
+      <c r="L340" s="1">
+        <v>56</v>
+      </c>
+      <c r="M340" s="1">
+        <v>1915</v>
+      </c>
+      <c r="N340" s="1">
+        <v>42</v>
+      </c>
+      <c r="O340" s="1">
+        <v>78</v>
+      </c>
+      <c r="P340" s="1">
+        <v>14</v>
+      </c>
+      <c r="T340" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="U340" s="1">
+        <v>54.8</v>
+      </c>
+    </row>
+    <row r="341" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B341" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C341" s="1">
+        <v>202301</v>
+      </c>
+      <c r="D341" s="1">
+        <v>162</v>
+      </c>
+      <c r="E341" s="1">
+        <v>138</v>
+      </c>
+      <c r="H341">
+        <v>57.349710000000002</v>
+      </c>
+      <c r="I341">
+        <v>-169.59164999999999</v>
+      </c>
+      <c r="J341" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L341" s="1">
+        <v>63</v>
+      </c>
+      <c r="M341" s="1">
+        <v>2914</v>
+      </c>
+      <c r="N341" s="1">
+        <v>76</v>
+      </c>
+      <c r="O341" s="1">
+        <v>28</v>
+      </c>
+      <c r="P341" s="1">
+        <v>18</v>
+      </c>
+      <c r="T341" s="1">
+        <v>7.2</v>
+      </c>
+      <c r="U341" s="1">
+        <v>47.5</v>
+      </c>
+    </row>
+    <row r="342" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="B342" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C342" s="1">
+        <v>202301</v>
+      </c>
+      <c r="D342" s="1">
+        <v>162</v>
+      </c>
+      <c r="E342" s="1">
+        <v>138</v>
+      </c>
+      <c r="H342">
+        <v>57.349710000000002</v>
+      </c>
+      <c r="I342">
+        <v>-169.59164999999999</v>
+      </c>
+      <c r="J342" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L342" s="1">
+        <v>58</v>
+      </c>
+      <c r="M342" s="1">
+        <v>2190</v>
+      </c>
+      <c r="N342" s="1">
+        <v>40</v>
+      </c>
+      <c r="O342" s="1">
+        <v>14</v>
+      </c>
+      <c r="P342" s="1">
+        <v>22</v>
+      </c>
+      <c r="T342" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="U342" s="1">
+        <v>30.5</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AB194">
     <sortCondition ref="C2:C194"/>
@@ -21128,7 +21316,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AA403"/>
+  <dimension ref="A1:AA401"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" style="1" customWidth="1"/>
@@ -40050,100 +40238,19 @@
       </c>
     </row>
     <row r="317" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="B317" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C317" s="1">
-        <v>202301</v>
-      </c>
-      <c r="D317" s="1">
-        <v>162</v>
-      </c>
-      <c r="E317" s="1">
-        <v>138</v>
-      </c>
-      <c r="G317">
-        <v>57.349710000000002</v>
-      </c>
-      <c r="H317">
-        <v>-169.59164999999999</v>
-      </c>
-      <c r="I317" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="K317" s="1">
-        <v>65</v>
-      </c>
-      <c r="L317" s="1">
-        <v>2936</v>
-      </c>
-      <c r="M317" s="1">
-        <v>68</v>
-      </c>
-      <c r="N317" s="1">
-        <v>86</v>
-      </c>
-      <c r="O317" s="1">
-        <v>30</v>
-      </c>
-      <c r="S317" s="1">
-        <v>4.7</v>
-      </c>
-      <c r="T317" s="1">
-        <v>51.3</v>
-      </c>
       <c r="AA317" s="1" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="318" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="B318" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C318" s="1">
-        <v>202301</v>
-      </c>
-      <c r="D318" s="1">
-        <v>162</v>
-      </c>
-      <c r="E318" s="1">
-        <v>138</v>
-      </c>
-      <c r="G318">
-        <v>57.349710000000002</v>
-      </c>
-      <c r="H318">
-        <v>-169.59164999999999</v>
-      </c>
-      <c r="I318" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="K318" s="1">
-        <v>56</v>
-      </c>
-      <c r="L318" s="1">
-        <v>1915</v>
-      </c>
-      <c r="M318" s="1">
-        <v>42</v>
-      </c>
-      <c r="N318" s="1">
-        <v>78</v>
-      </c>
-      <c r="O318" s="1">
-        <v>14</v>
-      </c>
-      <c r="S318" s="1">
-        <v>4.8</v>
-      </c>
-      <c r="T318" s="1">
-        <v>54.8</v>
-      </c>
       <c r="AA318" s="1" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="319" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A319" s="1">
+        <v>458</v>
+      </c>
       <c r="B319" s="1" t="s">
         <v>4</v>
       </c>
@@ -40154,43 +40261,46 @@
         <v>162</v>
       </c>
       <c r="E319" s="1">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="G319">
-        <v>57.349710000000002</v>
+        <v>56.338850000000001</v>
       </c>
       <c r="H319">
-        <v>-169.59164999999999</v>
+        <v>-170.05474000000001</v>
       </c>
       <c r="I319" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="J319">
+        <v>7</v>
+      </c>
       <c r="K319" s="1">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="L319" s="1">
-        <v>2914</v>
+        <v>1230</v>
       </c>
       <c r="M319" s="1">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="N319" s="1">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="O319" s="1">
         <v>18</v>
       </c>
       <c r="S319" s="1">
-        <v>7.2</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="T319" s="1">
-        <v>47.5</v>
-      </c>
-      <c r="AA319" s="1" t="s">
-        <v>78</v>
+        <v>81.3</v>
       </c>
     </row>
     <row r="320" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A320" s="1">
+        <v>459</v>
+      </c>
       <c r="B320" s="1" t="s">
         <v>4</v>
       </c>
@@ -40201,45 +40311,45 @@
         <v>162</v>
       </c>
       <c r="E320" s="1">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="G320">
-        <v>57.349710000000002</v>
+        <v>56.338850000000001</v>
       </c>
       <c r="H320">
-        <v>-169.59164999999999</v>
+        <v>-170.05474000000001</v>
       </c>
       <c r="I320" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="J320">
+        <v>8</v>
+      </c>
       <c r="K320" s="1">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="L320" s="1">
-        <v>2190</v>
+        <v>1100</v>
       </c>
       <c r="M320" s="1">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="N320" s="1">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="O320" s="1">
         <v>22</v>
       </c>
       <c r="S320" s="1">
-        <v>4.5</v>
+        <v>3.8</v>
       </c>
       <c r="T320" s="1">
-        <v>30.5</v>
-      </c>
-      <c r="AA320" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="321" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A321" s="1">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B321" s="1" t="s">
         <v>4</v>
@@ -40263,33 +40373,33 @@
         <v>3</v>
       </c>
       <c r="J321">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K321" s="1">
         <v>56</v>
       </c>
       <c r="L321" s="1">
-        <v>1230</v>
+        <v>1255</v>
       </c>
       <c r="M321" s="1">
-        <v>92</v>
+        <v>132</v>
       </c>
       <c r="N321" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O321" s="1">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="S321" s="1">
-        <v>4.5999999999999996</v>
+        <v>3.7</v>
       </c>
       <c r="T321" s="1">
-        <v>81.3</v>
+        <v>77.7</v>
       </c>
     </row>
     <row r="322" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A322" s="1">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B322" s="1" t="s">
         <v>4</v>
@@ -40313,33 +40423,33 @@
         <v>3</v>
       </c>
       <c r="J322">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K322" s="1">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="L322" s="1">
-        <v>1100</v>
+        <v>965</v>
       </c>
       <c r="M322" s="1">
-        <v>64</v>
+        <v>96</v>
       </c>
       <c r="N322" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O322" s="1">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="S322" s="1">
-        <v>3.8</v>
+        <v>5.5</v>
       </c>
       <c r="T322" s="1">
-        <v>76</v>
+        <v>81.2</v>
       </c>
     </row>
     <row r="323" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A323" s="1">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B323" s="1" t="s">
         <v>4</v>
@@ -40366,30 +40476,30 @@
         <v>9</v>
       </c>
       <c r="K323" s="1">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L323" s="1">
-        <v>1255</v>
+        <v>1420</v>
       </c>
       <c r="M323" s="1">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="N323" s="1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O323" s="1">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="S323" s="1">
-        <v>3.7</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="T323" s="1">
-        <v>77.7</v>
+        <v>78.900000000000006</v>
       </c>
     </row>
     <row r="324" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A324" s="1">
-        <v>461</v>
+        <v>480</v>
       </c>
       <c r="B324" s="1" t="s">
         <v>4</v>
@@ -40401,13 +40511,13 @@
         <v>162</v>
       </c>
       <c r="E324" s="1">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="G324">
-        <v>56.338850000000001</v>
+        <v>56.67915</v>
       </c>
       <c r="H324">
-        <v>-170.05474000000001</v>
+        <v>-170.14347000000001</v>
       </c>
       <c r="I324" s="1" t="s">
         <v>3</v>
@@ -40416,30 +40526,30 @@
         <v>9</v>
       </c>
       <c r="K324" s="1">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L324" s="1">
-        <v>965</v>
+        <v>998</v>
       </c>
       <c r="M324" s="1">
-        <v>96</v>
+        <v>66</v>
       </c>
       <c r="N324" s="1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O324" s="1">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="S324" s="1">
-        <v>5.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="T324" s="1">
-        <v>81.2</v>
+        <v>68</v>
       </c>
     </row>
     <row r="325" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A325" s="1">
-        <v>462</v>
+        <v>481</v>
       </c>
       <c r="B325" s="1" t="s">
         <v>4</v>
@@ -40451,45 +40561,45 @@
         <v>162</v>
       </c>
       <c r="E325" s="1">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="G325">
-        <v>56.338850000000001</v>
+        <v>56.67915</v>
       </c>
       <c r="H325">
-        <v>-170.05474000000001</v>
+        <v>-170.14347000000001</v>
       </c>
       <c r="I325" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J325">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K325" s="1">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="L325" s="1">
-        <v>1420</v>
+        <v>742</v>
       </c>
       <c r="M325" s="1">
-        <v>138</v>
+        <v>60</v>
       </c>
       <c r="N325" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O325" s="1">
-        <v>80</v>
+        <v>26</v>
       </c>
       <c r="S325" s="1">
-        <v>4.5999999999999996</v>
+        <v>5.2</v>
       </c>
       <c r="T325" s="1">
-        <v>78.900000000000006</v>
+        <v>75.2</v>
       </c>
     </row>
     <row r="326" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A326" s="1">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B326" s="1" t="s">
         <v>4</v>
@@ -40516,30 +40626,30 @@
         <v>9</v>
       </c>
       <c r="K326" s="1">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="L326" s="1">
-        <v>998</v>
+        <v>1186</v>
       </c>
       <c r="M326" s="1">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="N326" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O326" s="1">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="S326" s="1">
-        <v>4.9000000000000004</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="T326" s="1">
-        <v>68</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="327" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A327" s="1">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B327" s="1" t="s">
         <v>4</v>
@@ -40563,33 +40673,33 @@
         <v>3</v>
       </c>
       <c r="J327">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K327" s="1">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="L327" s="1">
-        <v>742</v>
+        <v>1188</v>
       </c>
       <c r="M327" s="1">
-        <v>60</v>
+        <v>96</v>
       </c>
       <c r="N327" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O327" s="1">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="S327" s="1">
-        <v>5.2</v>
+        <v>5.8</v>
       </c>
       <c r="T327" s="1">
-        <v>75.2</v>
+        <v>82.6</v>
       </c>
     </row>
     <row r="328" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A328" s="1">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B328" s="1" t="s">
         <v>4</v>
@@ -40616,30 +40726,30 @@
         <v>9</v>
       </c>
       <c r="K328" s="1">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="L328" s="1">
-        <v>1186</v>
+        <v>903</v>
       </c>
       <c r="M328" s="1">
-        <v>78</v>
+        <v>52</v>
       </c>
       <c r="N328" s="1">
         <v>2</v>
       </c>
       <c r="O328" s="1">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="S328" s="1">
-        <v>4.4000000000000004</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="T328" s="1">
-        <v>78.2</v>
+        <v>70.099999999999994</v>
       </c>
     </row>
     <row r="329" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A329" s="1">
-        <v>483</v>
+        <v>543</v>
       </c>
       <c r="B329" s="1" t="s">
         <v>4</v>
@@ -40651,45 +40761,45 @@
         <v>162</v>
       </c>
       <c r="E329" s="1">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="G329">
-        <v>56.67915</v>
+        <v>57.339010000000002</v>
       </c>
       <c r="H329">
-        <v>-170.14347000000001</v>
+        <v>-172.81381999999999</v>
       </c>
       <c r="I329" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J329">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K329" s="1">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="L329" s="1">
-        <v>1188</v>
+        <v>578</v>
       </c>
       <c r="M329" s="1">
-        <v>96</v>
+        <v>42</v>
       </c>
       <c r="N329" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O329" s="1">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="S329" s="1">
-        <v>5.8</v>
+        <v>4.8</v>
       </c>
       <c r="T329" s="1">
-        <v>82.6</v>
+        <v>73.599999999999994</v>
       </c>
     </row>
     <row r="330" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A330" s="1">
-        <v>484</v>
+        <v>544</v>
       </c>
       <c r="B330" s="1" t="s">
         <v>4</v>
@@ -40701,45 +40811,45 @@
         <v>162</v>
       </c>
       <c r="E330" s="1">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="G330">
-        <v>56.67915</v>
+        <v>57.339010000000002</v>
       </c>
       <c r="H330">
-        <v>-170.14347000000001</v>
+        <v>-172.81381999999999</v>
       </c>
       <c r="I330" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J330">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K330" s="1">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="L330" s="1">
-        <v>903</v>
+        <v>590</v>
       </c>
       <c r="M330" s="1">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="N330" s="1">
         <v>2</v>
       </c>
       <c r="O330" s="1">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="S330" s="1">
-        <v>4.9000000000000004</v>
+        <v>5.4</v>
       </c>
       <c r="T330" s="1">
-        <v>70.099999999999994</v>
+        <v>70.8</v>
       </c>
     </row>
     <row r="331" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A331" s="1">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="B331" s="1" t="s">
         <v>4</v>
@@ -40763,33 +40873,33 @@
         <v>3</v>
       </c>
       <c r="J331">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K331" s="1">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="L331" s="1">
-        <v>578</v>
+        <v>696</v>
       </c>
       <c r="M331" s="1">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="N331" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O331" s="1">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="S331" s="1">
-        <v>4.8</v>
+        <v>3.6</v>
       </c>
       <c r="T331" s="1">
-        <v>73.599999999999994</v>
+        <v>73.7</v>
       </c>
     </row>
     <row r="332" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A332" s="1">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B332" s="1" t="s">
         <v>4</v>
@@ -40813,33 +40923,33 @@
         <v>3</v>
       </c>
       <c r="J332">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K332" s="1">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="L332" s="1">
-        <v>590</v>
+        <v>1036</v>
       </c>
       <c r="M332" s="1">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="N332" s="1">
         <v>2</v>
       </c>
       <c r="O332" s="1">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="S332" s="1">
-        <v>5.4</v>
+        <v>3.8</v>
       </c>
       <c r="T332" s="1">
-        <v>70.8</v>
+        <v>72.3</v>
       </c>
     </row>
     <row r="333" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A333" s="1">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B333" s="1" t="s">
         <v>4</v>
@@ -40866,30 +40976,30 @@
         <v>5</v>
       </c>
       <c r="K333" s="1">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="L333" s="1">
-        <v>696</v>
+        <v>586</v>
       </c>
       <c r="M333" s="1">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="N333" s="1">
         <v>0</v>
       </c>
       <c r="O333" s="1">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="S333" s="1">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="T333" s="1">
-        <v>73.7</v>
+        <v>75.400000000000006</v>
       </c>
     </row>
     <row r="334" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A334" s="1">
-        <v>546</v>
+        <v>615</v>
       </c>
       <c r="B334" s="1" t="s">
         <v>4</v>
@@ -40901,45 +41011,45 @@
         <v>162</v>
       </c>
       <c r="E334" s="1">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="G334">
-        <v>57.339010000000002</v>
+        <v>61.000729999999997</v>
       </c>
       <c r="H334">
-        <v>-172.81381999999999</v>
+        <v>-172.79311000000001</v>
       </c>
       <c r="I334" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J334">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K334" s="1">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L334" s="1">
-        <v>1036</v>
+        <v>888</v>
       </c>
       <c r="M334" s="1">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="N334" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O334" s="1">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="S334" s="1">
-        <v>3.8</v>
+        <v>5</v>
       </c>
       <c r="T334" s="1">
-        <v>72.3</v>
+        <v>33.200000000000003</v>
       </c>
     </row>
     <row r="335" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A335" s="1">
-        <v>547</v>
+        <v>616</v>
       </c>
       <c r="B335" s="1" t="s">
         <v>4</v>
@@ -40951,45 +41061,45 @@
         <v>162</v>
       </c>
       <c r="E335" s="1">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="G335">
-        <v>57.339010000000002</v>
+        <v>61.000729999999997</v>
       </c>
       <c r="H335">
-        <v>-172.81381999999999</v>
+        <v>-172.79311000000001</v>
       </c>
       <c r="I335" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J335">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="K335" s="1">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="L335" s="1">
-        <v>586</v>
+        <v>702</v>
       </c>
       <c r="M335" s="1">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="N335" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O335" s="1">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="S335" s="1">
-        <v>3.4</v>
+        <v>4.8</v>
       </c>
       <c r="T335" s="1">
-        <v>75.400000000000006</v>
+        <v>60.3</v>
       </c>
     </row>
     <row r="336" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A336" s="1">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="B336" s="1" t="s">
         <v>4</v>
@@ -41013,33 +41123,33 @@
         <v>3</v>
       </c>
       <c r="J336">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K336" s="1">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="L336" s="1">
-        <v>888</v>
+        <v>450</v>
       </c>
       <c r="M336" s="1">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="N336" s="1">
         <v>0</v>
       </c>
       <c r="O336" s="1">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="S336" s="1">
-        <v>5</v>
+        <v>7.7</v>
       </c>
       <c r="T336" s="1">
-        <v>33.200000000000003</v>
+        <v>76.599999999999994</v>
       </c>
     </row>
     <row r="337" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A337" s="1">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="B337" s="1" t="s">
         <v>4</v>
@@ -41063,33 +41173,33 @@
         <v>3</v>
       </c>
       <c r="J337">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K337" s="1">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="L337" s="1">
-        <v>702</v>
+        <v>808</v>
       </c>
       <c r="M337" s="1">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="N337" s="1">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="O337" s="1">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="S337" s="1">
-        <v>4.8</v>
+        <v>3.4</v>
       </c>
       <c r="T337" s="1">
-        <v>60.3</v>
+        <v>46.3</v>
       </c>
     </row>
     <row r="338" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A338" s="1">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="B338" s="1" t="s">
         <v>4</v>
@@ -41113,33 +41223,33 @@
         <v>3</v>
       </c>
       <c r="J338">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K338" s="1">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="L338" s="1">
-        <v>450</v>
+        <v>646</v>
       </c>
       <c r="M338" s="1">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="N338" s="1">
         <v>0</v>
       </c>
       <c r="O338" s="1">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="S338" s="1">
-        <v>7.7</v>
+        <v>4</v>
       </c>
       <c r="T338" s="1">
-        <v>76.599999999999994</v>
+        <v>61.9</v>
       </c>
     </row>
     <row r="339" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A339" s="1">
-        <v>618</v>
+        <v>637</v>
       </c>
       <c r="B339" s="1" t="s">
         <v>4</v>
@@ -41151,45 +41261,45 @@
         <v>162</v>
       </c>
       <c r="E339" s="1">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="G339">
-        <v>61.000729999999997</v>
+        <v>60.185679999999998</v>
       </c>
       <c r="H339">
-        <v>-172.79311000000001</v>
+        <v>-173.03664000000001</v>
       </c>
       <c r="I339" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J339">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K339" s="1">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="L339" s="1">
-        <v>808</v>
+        <v>1675</v>
       </c>
       <c r="M339" s="1">
-        <v>18</v>
+        <v>80</v>
       </c>
       <c r="N339" s="1">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="O339" s="1">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="S339" s="1">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="T339" s="1">
-        <v>46.3</v>
+        <v>62.7</v>
       </c>
     </row>
     <row r="340" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A340" s="1">
-        <v>619</v>
+        <v>638</v>
       </c>
       <c r="B340" s="1" t="s">
         <v>4</v>
@@ -41201,45 +41311,45 @@
         <v>162</v>
       </c>
       <c r="E340" s="1">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="G340">
-        <v>61.000729999999997</v>
+        <v>60.185679999999998</v>
       </c>
       <c r="H340">
-        <v>-172.79311000000001</v>
+        <v>-173.03664000000001</v>
       </c>
       <c r="I340" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J340">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="K340" s="1">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="L340" s="1">
-        <v>646</v>
+        <v>1015</v>
       </c>
       <c r="M340" s="1">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="N340" s="1">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O340" s="1">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="S340" s="1">
-        <v>4</v>
+        <v>5.9</v>
       </c>
       <c r="T340" s="1">
-        <v>61.9</v>
+        <v>67</v>
       </c>
     </row>
     <row r="341" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A341" s="1">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="B341" s="1" t="s">
         <v>4</v>
@@ -41263,33 +41373,33 @@
         <v>3</v>
       </c>
       <c r="J341">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K341" s="1">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="L341" s="1">
-        <v>1675</v>
+        <v>795</v>
       </c>
       <c r="M341" s="1">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="N341" s="1">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="O341" s="1">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="S341" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T341" s="1">
-        <v>62.7</v>
+        <v>36.6</v>
       </c>
     </row>
     <row r="342" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A342" s="1">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="B342" s="1" t="s">
         <v>4</v>
@@ -41313,33 +41423,33 @@
         <v>3</v>
       </c>
       <c r="J342">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K342" s="1">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L342" s="1">
-        <v>1015</v>
+        <v>1205</v>
       </c>
       <c r="M342" s="1">
         <v>25</v>
       </c>
       <c r="N342" s="1">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="O342" s="1">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="S342" s="1">
-        <v>5.9</v>
+        <v>4.3</v>
       </c>
       <c r="T342" s="1">
-        <v>67</v>
+        <v>46.5</v>
       </c>
     </row>
     <row r="343" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A343" s="1">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="B343" s="1" t="s">
         <v>4</v>
@@ -41366,30 +41476,30 @@
         <v>8</v>
       </c>
       <c r="K343" s="1">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L343" s="1">
-        <v>795</v>
+        <v>1100</v>
       </c>
       <c r="M343" s="1">
         <v>30</v>
       </c>
       <c r="N343" s="1">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="O343" s="1">
         <v>15</v>
       </c>
       <c r="S343" s="1">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="T343" s="1">
-        <v>36.6</v>
+        <v>52.4</v>
       </c>
     </row>
     <row r="344" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A344" s="1">
-        <v>640</v>
+        <v>729</v>
       </c>
       <c r="B344" s="1" t="s">
         <v>4</v>
@@ -41401,45 +41511,45 @@
         <v>162</v>
       </c>
       <c r="E344" s="1">
-        <v>175</v>
+        <v>192</v>
       </c>
       <c r="G344">
-        <v>60.185679999999998</v>
+        <v>59.009799999999998</v>
       </c>
       <c r="H344">
-        <v>-173.03664000000001</v>
+        <v>-175.00677999999999</v>
       </c>
       <c r="I344" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J344">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="K344" s="1">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="L344" s="1">
-        <v>1205</v>
+        <v>1220</v>
       </c>
       <c r="M344" s="1">
-        <v>25</v>
+        <v>95</v>
       </c>
       <c r="N344" s="1">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="O344" s="1">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="S344" s="1">
-        <v>4.3</v>
+        <v>5.7</v>
       </c>
       <c r="T344" s="1">
-        <v>46.5</v>
+        <v>84.6</v>
       </c>
     </row>
     <row r="345" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A345" s="1">
-        <v>641</v>
+        <v>730</v>
       </c>
       <c r="B345" s="1" t="s">
         <v>4</v>
@@ -41451,45 +41561,45 @@
         <v>162</v>
       </c>
       <c r="E345" s="1">
-        <v>175</v>
+        <v>192</v>
       </c>
       <c r="G345">
-        <v>60.185679999999998</v>
+        <v>59.009799999999998</v>
       </c>
       <c r="H345">
-        <v>-173.03664000000001</v>
+        <v>-175.00677999999999</v>
       </c>
       <c r="I345" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J345">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K345" s="1">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="L345" s="1">
-        <v>1100</v>
+        <v>500</v>
       </c>
       <c r="M345" s="1">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="N345" s="1">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="O345" s="1">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="S345" s="1">
-        <v>4.3</v>
+        <v>6.6</v>
       </c>
       <c r="T345" s="1">
-        <v>52.4</v>
+        <v>75.900000000000006</v>
       </c>
     </row>
     <row r="346" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A346" s="1">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="B346" s="1" t="s">
         <v>4</v>
@@ -41513,33 +41623,33 @@
         <v>3</v>
       </c>
       <c r="J346">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K346" s="1">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="L346" s="1">
-        <v>1220</v>
+        <v>585</v>
       </c>
       <c r="M346" s="1">
-        <v>95</v>
+        <v>40</v>
       </c>
       <c r="N346" s="1">
         <v>5</v>
       </c>
       <c r="O346" s="1">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="S346" s="1">
-        <v>5.7</v>
+        <v>2.8</v>
       </c>
       <c r="T346" s="1">
-        <v>84.6</v>
+        <v>82.8</v>
       </c>
     </row>
     <row r="347" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A347" s="1">
-        <v>730</v>
+        <v>765</v>
       </c>
       <c r="B347" s="1" t="s">
         <v>4</v>
@@ -41551,45 +41661,45 @@
         <v>162</v>
       </c>
       <c r="E347" s="1">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="G347">
-        <v>59.009799999999998</v>
+        <v>60.002929999999999</v>
       </c>
       <c r="H347">
-        <v>-175.00677999999999</v>
+        <v>-177.93992</v>
       </c>
       <c r="I347" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J347">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K347" s="1">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="L347" s="1">
-        <v>500</v>
+        <v>1250</v>
       </c>
       <c r="M347" s="1">
-        <v>25</v>
+        <v>120</v>
       </c>
       <c r="N347" s="1">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="O347" s="1">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="S347" s="1">
-        <v>6.6</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="T347" s="1">
-        <v>75.900000000000006</v>
+        <v>84.1</v>
       </c>
     </row>
     <row r="348" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A348" s="1">
-        <v>731</v>
+        <v>766</v>
       </c>
       <c r="B348" s="1" t="s">
         <v>4</v>
@@ -41601,45 +41711,45 @@
         <v>162</v>
       </c>
       <c r="E348" s="1">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="G348">
-        <v>59.009799999999998</v>
+        <v>60.002929999999999</v>
       </c>
       <c r="H348">
-        <v>-175.00677999999999</v>
+        <v>-177.93992</v>
       </c>
       <c r="I348" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J348">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K348" s="1">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="L348" s="1">
-        <v>585</v>
+        <v>390</v>
       </c>
       <c r="M348" s="1">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="N348" s="1">
         <v>5</v>
       </c>
       <c r="O348" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S348" s="1">
-        <v>2.8</v>
+        <v>5.7</v>
       </c>
       <c r="T348" s="1">
-        <v>82.8</v>
+        <v>84.3</v>
       </c>
     </row>
     <row r="349" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A349" s="1">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="B349" s="1" t="s">
         <v>4</v>
@@ -41663,33 +41773,33 @@
         <v>3</v>
       </c>
       <c r="J349">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K349" s="1">
         <v>54</v>
       </c>
       <c r="L349" s="1">
-        <v>1250</v>
+        <v>1200</v>
       </c>
       <c r="M349" s="1">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="N349" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O349" s="1">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="S349" s="1">
-        <v>4.9000000000000004</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="T349" s="1">
-        <v>84.1</v>
+        <v>86.9</v>
       </c>
     </row>
     <row r="350" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A350" s="1">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="B350" s="1" t="s">
         <v>4</v>
@@ -41713,33 +41823,33 @@
         <v>3</v>
       </c>
       <c r="J350">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="K350" s="1">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="L350" s="1">
-        <v>390</v>
+        <v>805</v>
       </c>
       <c r="M350" s="1">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="N350" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O350" s="1">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="S350" s="1">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="T350" s="1">
-        <v>84.3</v>
+        <v>86.1</v>
       </c>
     </row>
     <row r="351" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A351" s="1">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="B351" s="1" t="s">
         <v>4</v>
@@ -41763,33 +41873,33 @@
         <v>3</v>
       </c>
       <c r="J351">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K351" s="1">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L351" s="1">
-        <v>1200</v>
+        <v>1030</v>
       </c>
       <c r="M351" s="1">
-        <v>130</v>
+        <v>80</v>
       </c>
       <c r="N351" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O351" s="1">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="S351" s="1">
         <v>4.5999999999999996</v>
       </c>
       <c r="T351" s="1">
-        <v>86.9</v>
+        <v>84</v>
       </c>
     </row>
     <row r="352" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A352" s="1">
-        <v>768</v>
+        <v>824</v>
       </c>
       <c r="B352" s="1" t="s">
         <v>4</v>
@@ -41801,45 +41911,45 @@
         <v>162</v>
       </c>
       <c r="E352" s="1">
-        <v>198</v>
+        <v>208</v>
       </c>
       <c r="G352">
-        <v>60.002929999999999</v>
+        <v>61.004399999999997</v>
       </c>
       <c r="H352">
-        <v>-177.93992</v>
+        <v>-175.55538999999999</v>
       </c>
       <c r="I352" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J352">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K352" s="1">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="L352" s="1">
-        <v>805</v>
+        <v>445</v>
       </c>
       <c r="M352" s="1">
-        <v>80</v>
+        <v>22</v>
       </c>
       <c r="N352" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O352" s="1">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="S352" s="1">
-        <v>5.9</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="T352" s="1">
-        <v>86.1</v>
+        <v>78.099999999999994</v>
       </c>
     </row>
     <row r="353" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A353" s="1">
-        <v>769</v>
+        <v>825</v>
       </c>
       <c r="B353" s="1" t="s">
         <v>4</v>
@@ -41851,45 +41961,45 @@
         <v>162</v>
       </c>
       <c r="E353" s="1">
-        <v>198</v>
+        <v>208</v>
       </c>
       <c r="G353">
-        <v>60.002929999999999</v>
+        <v>61.004399999999997</v>
       </c>
       <c r="H353">
-        <v>-177.93992</v>
+        <v>-175.55538999999999</v>
       </c>
       <c r="I353" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J353">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="K353" s="1">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="L353" s="1">
-        <v>1030</v>
+        <v>1425</v>
       </c>
       <c r="M353" s="1">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="N353" s="1">
         <v>2</v>
       </c>
       <c r="O353" s="1">
-        <v>26</v>
+        <v>138</v>
       </c>
       <c r="S353" s="1">
-        <v>4.5999999999999996</v>
+        <v>5.6</v>
       </c>
       <c r="T353" s="1">
-        <v>84</v>
+        <v>74.3</v>
       </c>
     </row>
     <row r="354" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A354" s="1">
-        <v>824</v>
+        <v>826</v>
       </c>
       <c r="B354" s="1" t="s">
         <v>4</v>
@@ -41913,33 +42023,33 @@
         <v>3</v>
       </c>
       <c r="J354">
+        <v>10</v>
+      </c>
+      <c r="K354" s="1">
+        <v>52</v>
+      </c>
+      <c r="L354" s="1">
+        <v>980</v>
+      </c>
+      <c r="M354" s="1">
+        <v>56</v>
+      </c>
+      <c r="N354" s="1">
+        <v>2</v>
+      </c>
+      <c r="O354" s="1">
+        <v>20</v>
+      </c>
+      <c r="S354" s="1">
         <v>5</v>
       </c>
-      <c r="K354" s="1">
-        <v>41</v>
-      </c>
-      <c r="L354" s="1">
-        <v>445</v>
-      </c>
-      <c r="M354" s="1">
-        <v>22</v>
-      </c>
-      <c r="N354" s="1">
-        <v>4</v>
-      </c>
-      <c r="O354" s="1">
-        <v>6</v>
-      </c>
-      <c r="S354" s="1">
-        <v>5.0999999999999996</v>
-      </c>
       <c r="T354" s="1">
-        <v>78.099999999999994</v>
+        <v>78.599999999999994</v>
       </c>
     </row>
     <row r="355" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A355" s="1">
-        <v>825</v>
+        <v>827</v>
       </c>
       <c r="B355" s="1" t="s">
         <v>4</v>
@@ -41963,33 +42073,33 @@
         <v>3</v>
       </c>
       <c r="J355">
+        <v>6</v>
+      </c>
+      <c r="K355" s="1">
+        <v>44</v>
+      </c>
+      <c r="L355" s="1">
+        <v>485</v>
+      </c>
+      <c r="M355" s="1">
+        <v>26</v>
+      </c>
+      <c r="N355" s="1">
         <v>8</v>
       </c>
-      <c r="K355" s="1">
-        <v>58</v>
-      </c>
-      <c r="L355" s="1">
-        <v>1425</v>
-      </c>
-      <c r="M355" s="1">
-        <v>64</v>
-      </c>
-      <c r="N355" s="1">
-        <v>2</v>
-      </c>
       <c r="O355" s="1">
-        <v>138</v>
+        <v>8</v>
       </c>
       <c r="S355" s="1">
-        <v>5.6</v>
+        <v>3.8</v>
       </c>
       <c r="T355" s="1">
-        <v>74.3</v>
+        <v>78</v>
       </c>
     </row>
     <row r="356" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A356" s="1">
-        <v>826</v>
+        <v>828</v>
       </c>
       <c r="B356" s="1" t="s">
         <v>4</v>
@@ -42013,33 +42123,33 @@
         <v>3</v>
       </c>
       <c r="J356">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K356" s="1">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="L356" s="1">
-        <v>980</v>
+        <v>340</v>
       </c>
       <c r="M356" s="1">
-        <v>56</v>
+        <v>16</v>
       </c>
       <c r="N356" s="1">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="O356" s="1">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="S356" s="1">
-        <v>5</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="T356" s="1">
-        <v>78.599999999999994</v>
+        <v>82.5</v>
       </c>
     </row>
     <row r="357" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A357" s="1">
-        <v>827</v>
+        <v>873</v>
       </c>
       <c r="B357" s="1" t="s">
         <v>4</v>
@@ -42051,45 +42161,45 @@
         <v>162</v>
       </c>
       <c r="E357" s="1">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="G357">
-        <v>61.004399999999997</v>
+        <v>61.335520000000002</v>
       </c>
       <c r="H357">
-        <v>-175.55538999999999</v>
+        <v>-176.30676</v>
       </c>
       <c r="I357" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J357">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="K357" s="1">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="L357" s="1">
-        <v>485</v>
+        <v>1500</v>
       </c>
       <c r="M357" s="1">
-        <v>26</v>
+        <v>172</v>
       </c>
       <c r="N357" s="1">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="O357" s="1">
-        <v>8</v>
+        <v>72</v>
       </c>
       <c r="S357" s="1">
-        <v>3.8</v>
+        <v>6.3</v>
       </c>
       <c r="T357" s="1">
-        <v>78</v>
+        <v>82.6</v>
       </c>
     </row>
     <row r="358" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A358" s="1">
-        <v>828</v>
+        <v>874</v>
       </c>
       <c r="B358" s="1" t="s">
         <v>4</v>
@@ -42101,45 +42211,45 @@
         <v>162</v>
       </c>
       <c r="E358" s="1">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="G358">
-        <v>61.004399999999997</v>
+        <v>61.335520000000002</v>
       </c>
       <c r="H358">
-        <v>-175.55538999999999</v>
+        <v>-176.30676</v>
       </c>
       <c r="I358" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J358">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K358" s="1">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="L358" s="1">
-        <v>340</v>
+        <v>870</v>
       </c>
       <c r="M358" s="1">
-        <v>16</v>
+        <v>90</v>
       </c>
       <c r="N358" s="1">
         <v>8</v>
       </c>
       <c r="O358" s="1">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="S358" s="1">
-        <v>8.8000000000000007</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="T358" s="1">
-        <v>82.5</v>
+        <v>79.900000000000006</v>
       </c>
     </row>
     <row r="359" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A359" s="1">
-        <v>873</v>
+        <v>875</v>
       </c>
       <c r="B359" s="1" t="s">
         <v>4</v>
@@ -42163,33 +42273,33 @@
         <v>3</v>
       </c>
       <c r="J359">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K359" s="1">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L359" s="1">
-        <v>1500</v>
+        <v>950</v>
       </c>
       <c r="M359" s="1">
-        <v>172</v>
+        <v>72</v>
       </c>
       <c r="N359" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O359" s="1">
-        <v>72</v>
+        <v>18</v>
       </c>
       <c r="S359" s="1">
-        <v>6.3</v>
+        <v>4.3</v>
       </c>
       <c r="T359" s="1">
-        <v>82.6</v>
+        <v>76.8</v>
       </c>
     </row>
     <row r="360" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A360" s="1">
-        <v>874</v>
+        <v>876</v>
       </c>
       <c r="B360" s="1" t="s">
         <v>4</v>
@@ -42213,33 +42323,33 @@
         <v>3</v>
       </c>
       <c r="J360">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K360" s="1">
         <v>49</v>
       </c>
       <c r="L360" s="1">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="M360" s="1">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="N360" s="1">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="O360" s="1">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="S360" s="1">
-        <v>4.5999999999999996</v>
+        <v>5.2</v>
       </c>
       <c r="T360" s="1">
-        <v>79.900000000000006</v>
+        <v>79</v>
       </c>
     </row>
     <row r="361" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A361" s="1">
-        <v>875</v>
+        <v>877</v>
       </c>
       <c r="B361" s="1" t="s">
         <v>4</v>
@@ -42263,101 +42373,101 @@
         <v>3</v>
       </c>
       <c r="J361">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K361" s="1">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="L361" s="1">
-        <v>950</v>
+        <v>1200</v>
       </c>
       <c r="M361" s="1">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="N361" s="1">
         <v>0</v>
       </c>
       <c r="O361" s="1">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="S361" s="1">
-        <v>4.3</v>
+        <v>5.7</v>
       </c>
       <c r="T361" s="1">
-        <v>76.8</v>
+        <v>77.2</v>
       </c>
     </row>
     <row r="362" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A362" s="1">
-        <v>876</v>
+        <v>8</v>
       </c>
       <c r="B362" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C362" s="1">
-        <v>202301</v>
+        <v>202302</v>
       </c>
       <c r="D362" s="1">
         <v>162</v>
       </c>
       <c r="E362" s="1">
-        <v>217</v>
+        <v>3</v>
       </c>
       <c r="G362">
-        <v>61.335520000000002</v>
+        <v>63.535240000000002</v>
       </c>
       <c r="H362">
-        <v>-176.30676</v>
+        <v>-171.99808999999999</v>
       </c>
       <c r="I362" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J362">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K362" s="1">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="L362" s="1">
-        <v>865</v>
+        <v>1200</v>
       </c>
       <c r="M362" s="1">
-        <v>82</v>
+        <v>60</v>
       </c>
       <c r="N362" s="1">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="O362" s="1">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="S362" s="1">
-        <v>5.2</v>
+        <v>3.5</v>
       </c>
       <c r="T362" s="1">
-        <v>79</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="363" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A363" s="1">
-        <v>877</v>
+        <v>9</v>
       </c>
       <c r="B363" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C363" s="1">
-        <v>202301</v>
+        <v>202302</v>
       </c>
       <c r="D363" s="1">
         <v>162</v>
       </c>
       <c r="E363" s="1">
-        <v>217</v>
+        <v>3</v>
       </c>
       <c r="G363">
-        <v>61.335520000000002</v>
+        <v>63.535240000000002</v>
       </c>
       <c r="H363">
-        <v>-176.30676</v>
+        <v>-171.99808999999999</v>
       </c>
       <c r="I363" s="1" t="s">
         <v>3</v>
@@ -42366,30 +42476,30 @@
         <v>11</v>
       </c>
       <c r="K363" s="1">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="L363" s="1">
-        <v>1200</v>
+        <v>1375</v>
       </c>
       <c r="M363" s="1">
-        <v>76</v>
+        <v>30</v>
       </c>
       <c r="N363" s="1">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="O363" s="1">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="S363" s="1">
-        <v>5.7</v>
+        <v>7.1</v>
       </c>
       <c r="T363" s="1">
-        <v>77.2</v>
+        <v>67.3</v>
       </c>
     </row>
     <row r="364" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A364" s="1">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B364" s="1" t="s">
         <v>4</v>
@@ -42416,31 +42526,28 @@
         <v>8</v>
       </c>
       <c r="K364" s="1">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="L364" s="1">
-        <v>1200</v>
+        <v>1140</v>
       </c>
       <c r="M364" s="1">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="N364" s="1">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="O364" s="1">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="S364" s="1">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="T364" s="1">
-        <v>53.3</v>
+        <v>61.3</v>
       </c>
     </row>
     <row r="365" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A365" s="1">
-        <v>9</v>
-      </c>
       <c r="B365" s="1" t="s">
         <v>4</v>
       </c>
@@ -42462,35 +42569,29 @@
       <c r="I365" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J365">
-        <v>11</v>
-      </c>
       <c r="K365" s="1">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="L365" s="1">
-        <v>1375</v>
+        <v>2030</v>
       </c>
       <c r="M365" s="1">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="N365" s="1">
-        <v>40</v>
+        <v>142</v>
       </c>
       <c r="O365" s="1">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="S365" s="1">
-        <v>7.1</v>
+        <v>3.8</v>
       </c>
       <c r="T365" s="1">
-        <v>67.3</v>
+        <v>44.3</v>
       </c>
     </row>
     <row r="366" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A366" s="1">
-        <v>10</v>
-      </c>
       <c r="B366" s="1" t="s">
         <v>4</v>
       </c>
@@ -42512,32 +42613,32 @@
       <c r="I366" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J366">
-        <v>8</v>
-      </c>
       <c r="K366" s="1">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="L366" s="1">
-        <v>1140</v>
+        <v>1676</v>
       </c>
       <c r="M366" s="1">
-        <v>40</v>
+        <v>82</v>
       </c>
       <c r="N366" s="1">
-        <v>34</v>
+        <v>114</v>
       </c>
       <c r="O366" s="1">
-        <v>20</v>
+        <v>134</v>
       </c>
       <c r="S366" s="1">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="T366" s="1">
-        <v>61.3</v>
+        <v>41.7</v>
       </c>
     </row>
     <row r="367" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A367" s="1">
+        <v>21</v>
+      </c>
       <c r="B367" s="1" t="s">
         <v>4</v>
       </c>
@@ -42548,40 +42649,46 @@
         <v>162</v>
       </c>
       <c r="E367" s="1">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G367">
-        <v>63.535240000000002</v>
+        <v>63.662579999999998</v>
       </c>
       <c r="H367">
-        <v>-171.99808999999999</v>
+        <v>-169.79001</v>
       </c>
       <c r="I367" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="J367" s="1">
+        <v>12</v>
+      </c>
       <c r="K367" s="1">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="L367" s="1">
-        <v>2030</v>
+        <v>1110</v>
       </c>
       <c r="M367" s="1">
-        <v>90</v>
+        <v>52</v>
       </c>
       <c r="N367" s="1">
-        <v>142</v>
+        <v>2</v>
       </c>
       <c r="O367" s="1">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="S367" s="1">
         <v>3.8</v>
       </c>
       <c r="T367" s="1">
-        <v>44.3</v>
+        <v>60</v>
       </c>
     </row>
     <row r="368" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A368" s="1">
+        <v>23</v>
+      </c>
       <c r="B368" s="1" t="s">
         <v>4</v>
       </c>
@@ -42592,43 +42699,43 @@
         <v>162</v>
       </c>
       <c r="E368" s="1">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G368">
-        <v>63.535240000000002</v>
+        <v>63.662579999999998</v>
       </c>
       <c r="H368">
-        <v>-171.99808999999999</v>
+        <v>-169.79001</v>
       </c>
       <c r="I368" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="J368" s="1">
+        <v>13</v>
+      </c>
       <c r="K368" s="1">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="L368" s="1">
-        <v>1676</v>
+        <v>2276</v>
       </c>
       <c r="M368" s="1">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="N368" s="1">
-        <v>114</v>
+        <v>6</v>
       </c>
       <c r="O368" s="1">
-        <v>134</v>
+        <v>56</v>
       </c>
       <c r="S368" s="1">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="T368" s="1">
-        <v>41.7</v>
+        <v>44.3</v>
       </c>
     </row>
     <row r="369" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A369" s="1">
-        <v>21</v>
-      </c>
       <c r="B369" s="1" t="s">
         <v>4</v>
       </c>
@@ -42650,35 +42757,29 @@
       <c r="I369" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J369" s="1">
-        <v>12</v>
-      </c>
       <c r="K369" s="1">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="L369" s="1">
-        <v>1110</v>
+        <v>1980</v>
       </c>
       <c r="M369" s="1">
-        <v>52</v>
+        <v>116</v>
       </c>
       <c r="N369" s="1">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="O369" s="1">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="S369" s="1">
-        <v>3.8</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="T369" s="1">
-        <v>60</v>
+        <v>61.8</v>
       </c>
     </row>
     <row r="370" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A370" s="1">
-        <v>23</v>
-      </c>
       <c r="B370" s="1" t="s">
         <v>4</v>
       </c>
@@ -42700,32 +42801,32 @@
       <c r="I370" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J370" s="1">
-        <v>13</v>
-      </c>
       <c r="K370" s="1">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="L370" s="1">
-        <v>2276</v>
+        <v>2250</v>
       </c>
       <c r="M370" s="1">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="N370" s="1">
-        <v>6</v>
+        <v>96</v>
       </c>
       <c r="O370" s="1">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="S370" s="1">
-        <v>4.3</v>
+        <v>3.7</v>
       </c>
       <c r="T370" s="1">
-        <v>44.3</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="371" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A371" s="1">
+        <v>58</v>
+      </c>
       <c r="B371" s="1" t="s">
         <v>4</v>
       </c>
@@ -42736,40 +42837,46 @@
         <v>162</v>
       </c>
       <c r="E371" s="1">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="G371">
-        <v>63.662579999999998</v>
+        <v>65.002970000000005</v>
       </c>
       <c r="H371">
-        <v>-169.79001</v>
+        <v>-169.15404000000001</v>
       </c>
       <c r="I371" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="J371">
+        <v>11</v>
+      </c>
       <c r="K371" s="1">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="L371" s="1">
-        <v>1980</v>
+        <v>1490</v>
       </c>
       <c r="M371" s="1">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="N371" s="1">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="O371" s="1">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="S371" s="1">
-        <v>4.0999999999999996</v>
+        <v>4.3</v>
       </c>
       <c r="T371" s="1">
-        <v>61.8</v>
+        <v>51</v>
       </c>
     </row>
     <row r="372" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A372" s="1">
+        <v>59</v>
+      </c>
       <c r="B372" s="1" t="s">
         <v>4</v>
       </c>
@@ -42780,42 +42887,45 @@
         <v>162</v>
       </c>
       <c r="E372" s="1">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="G372">
-        <v>63.662579999999998</v>
+        <v>65.002970000000005</v>
       </c>
       <c r="H372">
-        <v>-169.79001</v>
+        <v>-169.15404000000001</v>
       </c>
       <c r="I372" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="J372">
+        <v>11</v>
+      </c>
       <c r="K372" s="1">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="L372" s="1">
-        <v>2250</v>
+        <v>1195</v>
       </c>
       <c r="M372" s="1">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="N372" s="1">
-        <v>96</v>
+        <v>6</v>
       </c>
       <c r="O372" s="1">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="S372" s="1">
-        <v>3.7</v>
+        <v>4.3</v>
       </c>
       <c r="T372" s="1">
-        <v>37.5</v>
+        <v>73.8</v>
       </c>
     </row>
     <row r="373" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A373" s="1">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B373" s="1" t="s">
         <v>4</v>
@@ -42839,34 +42949,31 @@
         <v>3</v>
       </c>
       <c r="J373">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="K373" s="1">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="L373" s="1">
-        <v>1490</v>
+        <v>1220</v>
       </c>
       <c r="M373" s="1">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="N373" s="1">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="O373" s="1">
         <v>28</v>
       </c>
       <c r="S373" s="1">
-        <v>4.3</v>
+        <v>4</v>
       </c>
       <c r="T373" s="1">
-        <v>51</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="374" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A374" s="1">
-        <v>59</v>
-      </c>
       <c r="B374" s="1" t="s">
         <v>4</v>
       </c>
@@ -42888,35 +42995,29 @@
       <c r="I374" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J374">
-        <v>11</v>
-      </c>
       <c r="K374" s="1">
         <v>56</v>
       </c>
       <c r="L374" s="1">
-        <v>1195</v>
+        <v>1245</v>
       </c>
       <c r="M374" s="1">
-        <v>96</v>
+        <v>58</v>
       </c>
       <c r="N374" s="1">
-        <v>6</v>
+        <v>56</v>
       </c>
       <c r="O374" s="1">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="S374" s="1">
-        <v>4.3</v>
+        <v>4.8</v>
       </c>
       <c r="T374" s="1">
-        <v>73.8</v>
+        <v>60.3</v>
       </c>
     </row>
     <row r="375" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A375" s="1">
-        <v>60</v>
-      </c>
       <c r="B375" s="1" t="s">
         <v>4</v>
       </c>
@@ -42938,32 +43039,32 @@
       <c r="I375" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J375">
-        <v>18</v>
-      </c>
       <c r="K375" s="1">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="L375" s="1">
-        <v>1220</v>
+        <v>1400</v>
       </c>
       <c r="M375" s="1">
-        <v>56</v>
+        <v>98</v>
       </c>
       <c r="N375" s="1">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="O375" s="1">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="S375" s="1">
-        <v>4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="T375" s="1">
-        <v>53.3</v>
+        <v>60.5</v>
       </c>
     </row>
     <row r="376" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A376" s="1">
+        <v>99</v>
+      </c>
       <c r="B376" s="1" t="s">
         <v>4</v>
       </c>
@@ -42974,40 +43075,46 @@
         <v>162</v>
       </c>
       <c r="E376" s="1">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="G376">
-        <v>65.002970000000005</v>
+        <v>64.339230000000001</v>
       </c>
       <c r="H376">
-        <v>-169.15404000000001</v>
+        <v>-168.33761000000001</v>
       </c>
       <c r="I376" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="J376">
+        <v>12</v>
+      </c>
       <c r="K376" s="1">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="L376" s="1">
-        <v>1245</v>
+        <v>1505</v>
       </c>
       <c r="M376" s="1">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="N376" s="1">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="O376" s="1">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="S376" s="1">
-        <v>4.8</v>
+        <v>3.8</v>
       </c>
       <c r="T376" s="1">
-        <v>60.3</v>
+        <v>36</v>
       </c>
     </row>
     <row r="377" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A377" s="1">
+        <v>100</v>
+      </c>
       <c r="B377" s="1" t="s">
         <v>4</v>
       </c>
@@ -43018,42 +43125,45 @@
         <v>162</v>
       </c>
       <c r="E377" s="1">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="G377">
-        <v>65.002970000000005</v>
+        <v>64.339230000000001</v>
       </c>
       <c r="H377">
-        <v>-169.15404000000001</v>
+        <v>-168.33761000000001</v>
       </c>
       <c r="I377" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="J377">
+        <v>10</v>
+      </c>
       <c r="K377" s="1">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="L377" s="1">
-        <v>1400</v>
+        <v>1740</v>
       </c>
       <c r="M377" s="1">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="N377" s="1">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="O377" s="1">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="S377" s="1">
-        <v>4.4000000000000004</v>
+        <v>5</v>
       </c>
       <c r="T377" s="1">
-        <v>60.5</v>
+        <v>58.6</v>
       </c>
     </row>
     <row r="378" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A378" s="1">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B378" s="1" t="s">
         <v>4</v>
@@ -43077,34 +43187,31 @@
         <v>3</v>
       </c>
       <c r="J378">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="K378" s="1">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L378" s="1">
-        <v>1505</v>
+        <v>1515</v>
       </c>
       <c r="M378" s="1">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="N378" s="1">
-        <v>76</v>
+        <v>2</v>
       </c>
       <c r="O378" s="1">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="S378" s="1">
-        <v>3.8</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="T378" s="1">
-        <v>36</v>
+        <v>65.900000000000006</v>
       </c>
     </row>
     <row r="379" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A379" s="1">
-        <v>100</v>
-      </c>
       <c r="B379" s="1" t="s">
         <v>4</v>
       </c>
@@ -43126,35 +43233,29 @@
       <c r="I379" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J379">
-        <v>10</v>
-      </c>
       <c r="K379" s="1">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="L379" s="1">
-        <v>1740</v>
+        <v>1610</v>
       </c>
       <c r="M379" s="1">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="N379" s="1">
         <v>0</v>
       </c>
       <c r="O379" s="1">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="S379" s="1">
-        <v>5</v>
+        <v>3.9</v>
       </c>
       <c r="T379" s="1">
-        <v>58.6</v>
+        <v>45.7</v>
       </c>
     </row>
     <row r="380" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A380" s="1">
-        <v>101</v>
-      </c>
       <c r="B380" s="1" t="s">
         <v>4</v>
       </c>
@@ -43176,32 +43277,32 @@
       <c r="I380" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J380">
-        <v>9</v>
-      </c>
       <c r="K380" s="1">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L380" s="1">
-        <v>1515</v>
+        <v>1810</v>
       </c>
       <c r="M380" s="1">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="N380" s="1">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="O380" s="1">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="S380" s="1">
-        <v>4.5999999999999996</v>
+        <v>3.9</v>
       </c>
       <c r="T380" s="1">
-        <v>65.900000000000006</v>
+        <v>54.8</v>
       </c>
     </row>
     <row r="381" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A381" s="1">
+        <v>126</v>
+      </c>
       <c r="B381" s="1" t="s">
         <v>4</v>
       </c>
@@ -43212,40 +43313,46 @@
         <v>162</v>
       </c>
       <c r="E381" s="1">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="G381">
-        <v>64.339230000000001</v>
+        <v>62.99521</v>
       </c>
       <c r="H381">
-        <v>-168.33761000000001</v>
+        <v>-171.10216</v>
       </c>
       <c r="I381" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="J381">
+        <v>9</v>
+      </c>
       <c r="K381" s="1">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="L381" s="1">
-        <v>1610</v>
+        <v>1054</v>
       </c>
       <c r="M381" s="1">
-        <v>106</v>
+        <v>56</v>
       </c>
       <c r="N381" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O381" s="1">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="S381" s="1">
-        <v>3.9</v>
+        <v>6.4</v>
       </c>
       <c r="T381" s="1">
-        <v>45.7</v>
+        <v>73.599999999999994</v>
       </c>
     </row>
     <row r="382" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A382" s="1">
+        <v>127</v>
+      </c>
       <c r="B382" s="1" t="s">
         <v>4</v>
       </c>
@@ -43256,42 +43363,45 @@
         <v>162</v>
       </c>
       <c r="E382" s="1">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="G382">
-        <v>64.339230000000001</v>
+        <v>62.99521</v>
       </c>
       <c r="H382">
-        <v>-168.33761000000001</v>
+        <v>-171.10216</v>
       </c>
       <c r="I382" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="J382">
+        <v>9</v>
+      </c>
       <c r="K382" s="1">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="L382" s="1">
-        <v>1810</v>
+        <v>1190</v>
       </c>
       <c r="M382" s="1">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="N382" s="1">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="O382" s="1">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="S382" s="1">
         <v>3.9</v>
       </c>
       <c r="T382" s="1">
-        <v>54.8</v>
+        <v>71.7</v>
       </c>
     </row>
     <row r="383" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A383" s="1">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B383" s="1" t="s">
         <v>4</v>
@@ -43321,27 +43431,27 @@
         <v>58</v>
       </c>
       <c r="L383" s="1">
-        <v>1054</v>
+        <v>1088</v>
       </c>
       <c r="M383" s="1">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="N383" s="1">
         <v>2</v>
       </c>
       <c r="O383" s="1">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="S383" s="1">
-        <v>6.4</v>
+        <v>6</v>
       </c>
       <c r="T383" s="1">
-        <v>73.599999999999994</v>
+        <v>60.6</v>
       </c>
     </row>
     <row r="384" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A384" s="1">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="B384" s="1" t="s">
         <v>4</v>
@@ -43353,45 +43463,45 @@
         <v>162</v>
       </c>
       <c r="E384" s="1">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="G384">
-        <v>62.99521</v>
+        <v>63.010440000000003</v>
       </c>
       <c r="H384">
-        <v>-171.10216</v>
+        <v>-174.01429999999999</v>
       </c>
       <c r="I384" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J384">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K384" s="1">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L384" s="1">
-        <v>1190</v>
+        <v>1102</v>
       </c>
       <c r="M384" s="1">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="N384" s="1">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="O384" s="1">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="S384" s="1">
-        <v>3.9</v>
+        <v>6.5</v>
       </c>
       <c r="T384" s="1">
-        <v>71.7</v>
+        <v>72.7</v>
       </c>
     </row>
     <row r="385" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A385" s="1">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="B385" s="1" t="s">
         <v>4</v>
@@ -43403,45 +43513,45 @@
         <v>162</v>
       </c>
       <c r="E385" s="1">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="G385">
-        <v>62.99521</v>
+        <v>63.010440000000003</v>
       </c>
       <c r="H385">
-        <v>-171.10216</v>
+        <v>-174.01429999999999</v>
       </c>
       <c r="I385" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J385">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="K385" s="1">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="L385" s="1">
-        <v>1088</v>
+        <v>1046</v>
       </c>
       <c r="M385" s="1">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="N385" s="1">
-        <v>2</v>
+        <v>66</v>
       </c>
       <c r="O385" s="1">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="S385" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="T385" s="1">
-        <v>60.6</v>
+        <v>40.799999999999997</v>
       </c>
     </row>
     <row r="386" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A386" s="1">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B386" s="1" t="s">
         <v>4</v>
@@ -43465,33 +43575,33 @@
         <v>3</v>
       </c>
       <c r="J386">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K386" s="1">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L386" s="1">
-        <v>1102</v>
+        <v>882</v>
       </c>
       <c r="M386" s="1">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="N386" s="1">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="O386" s="1">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="S386" s="1">
-        <v>6.5</v>
+        <v>5.9</v>
       </c>
       <c r="T386" s="1">
-        <v>72.7</v>
+        <v>73</v>
       </c>
     </row>
     <row r="387" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A387" s="1">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="B387" s="1" t="s">
         <v>4</v>
@@ -43503,45 +43613,45 @@
         <v>162</v>
       </c>
       <c r="E387" s="1">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="G387">
-        <v>63.010440000000003</v>
+        <v>62.332459999999998</v>
       </c>
       <c r="H387">
-        <v>-174.01429999999999</v>
+        <v>-172.44681</v>
       </c>
       <c r="I387" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J387">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="K387" s="1">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="L387" s="1">
-        <v>1046</v>
+        <v>712</v>
       </c>
       <c r="M387" s="1">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="N387" s="1">
-        <v>66</v>
+        <v>2</v>
       </c>
       <c r="O387" s="1">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="S387" s="1">
-        <v>8</v>
+        <v>3.8</v>
       </c>
       <c r="T387" s="1">
-        <v>40.799999999999997</v>
+        <v>86.5</v>
       </c>
     </row>
     <row r="388" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A388" s="1">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="B388" s="1" t="s">
         <v>4</v>
@@ -43553,45 +43663,45 @@
         <v>162</v>
       </c>
       <c r="E388" s="1">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="G388">
-        <v>63.010440000000003</v>
+        <v>62.332459999999998</v>
       </c>
       <c r="H388">
-        <v>-174.01429999999999</v>
+        <v>-172.44681</v>
       </c>
       <c r="I388" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J388">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K388" s="1">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="L388" s="1">
-        <v>882</v>
+        <v>696</v>
       </c>
       <c r="M388" s="1">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="N388" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O388" s="1">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="S388" s="1">
-        <v>5.9</v>
+        <v>4.7</v>
       </c>
       <c r="T388" s="1">
-        <v>73</v>
+        <v>78.400000000000006</v>
       </c>
     </row>
     <row r="389" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A389" s="1">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B389" s="1" t="s">
         <v>4</v>
@@ -43615,34 +43725,31 @@
         <v>3</v>
       </c>
       <c r="J389">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K389" s="1">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="L389" s="1">
-        <v>712</v>
+        <v>612</v>
       </c>
       <c r="M389" s="1">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="N389" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O389" s="1">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="S389" s="1">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="T389" s="1">
-        <v>86.5</v>
+        <v>79.3</v>
       </c>
     </row>
     <row r="390" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A390" s="1">
-        <v>158</v>
-      </c>
       <c r="B390" s="1" t="s">
         <v>4</v>
       </c>
@@ -43664,35 +43771,29 @@
       <c r="I390" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J390">
-        <v>9</v>
-      </c>
       <c r="K390" s="1">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="L390" s="1">
-        <v>696</v>
+        <v>842</v>
       </c>
       <c r="M390" s="1">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="N390" s="1">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="O390" s="1">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="S390" s="1">
-        <v>4.7</v>
+        <v>4</v>
       </c>
       <c r="T390" s="1">
-        <v>78.400000000000006</v>
+        <v>76.900000000000006</v>
       </c>
     </row>
     <row r="391" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A391" s="1">
-        <v>159</v>
-      </c>
       <c r="B391" s="1" t="s">
         <v>4</v>
       </c>
@@ -43714,32 +43815,32 @@
       <c r="I391" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J391">
-        <v>6</v>
-      </c>
       <c r="K391" s="1">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="L391" s="1">
-        <v>612</v>
+        <v>712</v>
       </c>
       <c r="M391" s="1">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="N391" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O391" s="1">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="S391" s="1">
-        <v>4</v>
+        <v>3.3</v>
       </c>
       <c r="T391" s="1">
-        <v>79.3</v>
+        <v>74.7</v>
       </c>
     </row>
     <row r="392" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A392" s="1">
+        <v>192</v>
+      </c>
       <c r="B392" s="1" t="s">
         <v>4</v>
       </c>
@@ -43750,40 +43851,46 @@
         <v>162</v>
       </c>
       <c r="E392" s="1">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G392">
-        <v>62.332459999999998</v>
+        <v>61.33587</v>
       </c>
       <c r="H392">
-        <v>-172.44681</v>
+        <v>-172.95796999999999</v>
       </c>
       <c r="I392" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="J392">
+        <v>7</v>
+      </c>
       <c r="K392" s="1">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="L392" s="1">
-        <v>842</v>
+        <v>762</v>
       </c>
       <c r="M392" s="1">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="N392" s="1">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="O392" s="1">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="S392" s="1">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="T392" s="1">
-        <v>76.900000000000006</v>
+        <v>73.400000000000006</v>
       </c>
     </row>
     <row r="393" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A393" s="1">
+        <v>193</v>
+      </c>
       <c r="B393" s="1" t="s">
         <v>4</v>
       </c>
@@ -43794,42 +43901,45 @@
         <v>162</v>
       </c>
       <c r="E393" s="1">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G393">
-        <v>62.332459999999998</v>
+        <v>61.33587</v>
       </c>
       <c r="H393">
-        <v>-172.44681</v>
+        <v>-172.95796999999999</v>
       </c>
       <c r="I393" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="J393">
+        <v>13</v>
+      </c>
       <c r="K393" s="1">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="L393" s="1">
-        <v>712</v>
+        <v>1208</v>
       </c>
       <c r="M393" s="1">
-        <v>34</v>
+        <v>76</v>
       </c>
       <c r="N393" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O393" s="1">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="S393" s="1">
-        <v>3.3</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="T393" s="1">
-        <v>74.7</v>
+        <v>65.599999999999994</v>
       </c>
     </row>
     <row r="394" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A394" s="1">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B394" s="1" t="s">
         <v>4</v>
@@ -43853,34 +43963,31 @@
         <v>3</v>
       </c>
       <c r="J394">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="K394" s="1">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="L394" s="1">
-        <v>762</v>
+        <v>1336</v>
       </c>
       <c r="M394" s="1">
-        <v>36</v>
+        <v>102</v>
       </c>
       <c r="N394" s="1">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="O394" s="1">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="S394" s="1">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
       <c r="T394" s="1">
-        <v>73.400000000000006</v>
+        <v>77.400000000000006</v>
       </c>
     </row>
     <row r="395" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A395" s="1">
-        <v>193</v>
-      </c>
       <c r="B395" s="1" t="s">
         <v>4</v>
       </c>
@@ -43902,35 +44009,29 @@
       <c r="I395" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J395">
-        <v>13</v>
-      </c>
       <c r="K395" s="1">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L395" s="1">
-        <v>1208</v>
+        <v>982</v>
       </c>
       <c r="M395" s="1">
-        <v>76</v>
+        <v>44</v>
       </c>
       <c r="N395" s="1">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="O395" s="1">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="S395" s="1">
-        <v>4.9000000000000004</v>
+        <v>4.8</v>
       </c>
       <c r="T395" s="1">
-        <v>65.599999999999994</v>
+        <v>67.3</v>
       </c>
     </row>
     <row r="396" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A396" s="1">
-        <v>194</v>
-      </c>
       <c r="B396" s="1" t="s">
         <v>4</v>
       </c>
@@ -43952,32 +44053,32 @@
       <c r="I396" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J396">
-        <v>12</v>
-      </c>
       <c r="K396" s="1">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="L396" s="1">
-        <v>1336</v>
+        <v>862</v>
       </c>
       <c r="M396" s="1">
-        <v>102</v>
+        <v>52</v>
       </c>
       <c r="N396" s="1">
+        <v>6</v>
+      </c>
+      <c r="O396" s="1">
         <v>16</v>
       </c>
-      <c r="O396" s="1">
-        <v>40</v>
-      </c>
       <c r="S396" s="1">
-        <v>4.2</v>
+        <v>3.8</v>
       </c>
       <c r="T396" s="1">
-        <v>77.400000000000006</v>
+        <v>86</v>
       </c>
     </row>
     <row r="397" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A397" s="1">
+        <v>228</v>
+      </c>
       <c r="B397" s="1" t="s">
         <v>4</v>
       </c>
@@ -43988,40 +44089,46 @@
         <v>162</v>
       </c>
       <c r="E397" s="1">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="G397">
-        <v>61.33587</v>
+        <v>60.669910000000002</v>
       </c>
       <c r="H397">
-        <v>-172.95796999999999</v>
+        <v>-170.07918000000001</v>
       </c>
       <c r="I397" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="J397">
+        <v>7</v>
+      </c>
       <c r="K397" s="1">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="L397" s="1">
-        <v>982</v>
+        <v>902</v>
       </c>
       <c r="M397" s="1">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="N397" s="1">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="O397" s="1">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="S397" s="1">
-        <v>4.8</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="T397" s="1">
-        <v>67.3</v>
+        <v>77.7</v>
       </c>
     </row>
     <row r="398" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A398" s="1">
+        <v>229</v>
+      </c>
       <c r="B398" s="1" t="s">
         <v>4</v>
       </c>
@@ -44032,42 +44139,45 @@
         <v>162</v>
       </c>
       <c r="E398" s="1">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="G398">
-        <v>61.33587</v>
+        <v>60.669910000000002</v>
       </c>
       <c r="H398">
-        <v>-172.95796999999999</v>
+        <v>-170.07918000000001</v>
       </c>
       <c r="I398" s="1" t="s">
         <v>3</v>
+      </c>
+      <c r="J398">
+        <v>9</v>
       </c>
       <c r="K398" s="1">
         <v>52</v>
       </c>
       <c r="L398" s="1">
-        <v>862</v>
+        <v>822</v>
       </c>
       <c r="M398" s="1">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="N398" s="1">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O398" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="S398" s="1">
-        <v>3.8</v>
+        <v>5.3</v>
       </c>
       <c r="T398" s="1">
-        <v>86</v>
+        <v>76.900000000000006</v>
       </c>
     </row>
     <row r="399" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A399" s="1">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B399" s="1" t="s">
         <v>4</v>
@@ -44091,34 +44201,31 @@
         <v>3</v>
       </c>
       <c r="J399">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K399" s="1">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="L399" s="1">
-        <v>902</v>
+        <v>972</v>
       </c>
       <c r="M399" s="1">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="N399" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O399" s="1">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="S399" s="1">
-        <v>4.9000000000000004</v>
+        <v>5.7</v>
       </c>
       <c r="T399" s="1">
-        <v>77.7</v>
+        <v>70.099999999999994</v>
       </c>
     </row>
     <row r="400" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A400" s="1">
-        <v>229</v>
-      </c>
       <c r="B400" s="1" t="s">
         <v>4</v>
       </c>
@@ -44140,35 +44247,29 @@
       <c r="I400" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J400">
-        <v>9</v>
-      </c>
       <c r="K400" s="1">
         <v>52</v>
       </c>
       <c r="L400" s="1">
-        <v>822</v>
+        <v>1002</v>
       </c>
       <c r="M400" s="1">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="N400" s="1">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="O400" s="1">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="S400" s="1">
-        <v>5.3</v>
+        <v>4</v>
       </c>
       <c r="T400" s="1">
-        <v>76.900000000000006</v>
-      </c>
-    </row>
-    <row r="401" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A401" s="1">
-        <v>230</v>
-      </c>
+        <v>78.7</v>
+      </c>
+    </row>
+    <row r="401" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B401" s="1" t="s">
         <v>4</v>
       </c>
@@ -44190,116 +44291,25 @@
       <c r="I401" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J401">
-        <v>9</v>
-      </c>
       <c r="K401" s="1">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="L401" s="1">
-        <v>972</v>
+        <v>868</v>
       </c>
       <c r="M401" s="1">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="N401" s="1">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O401" s="1">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="S401" s="1">
-        <v>5.7</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="T401" s="1">
-        <v>70.099999999999994</v>
-      </c>
-    </row>
-    <row r="402" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="B402" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C402" s="1">
-        <v>202302</v>
-      </c>
-      <c r="D402" s="1">
-        <v>162</v>
-      </c>
-      <c r="E402" s="1">
-        <v>66</v>
-      </c>
-      <c r="G402">
-        <v>60.669910000000002</v>
-      </c>
-      <c r="H402">
-        <v>-170.07918000000001</v>
-      </c>
-      <c r="I402" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="K402" s="1">
-        <v>52</v>
-      </c>
-      <c r="L402" s="1">
-        <v>1002</v>
-      </c>
-      <c r="M402" s="1">
-        <v>76</v>
-      </c>
-      <c r="N402" s="1">
-        <v>8</v>
-      </c>
-      <c r="O402" s="1">
-        <v>28</v>
-      </c>
-      <c r="S402" s="1">
-        <v>4</v>
-      </c>
-      <c r="T402" s="1">
-        <v>78.7</v>
-      </c>
-    </row>
-    <row r="403" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="B403" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C403" s="1">
-        <v>202302</v>
-      </c>
-      <c r="D403" s="1">
-        <v>162</v>
-      </c>
-      <c r="E403" s="1">
-        <v>66</v>
-      </c>
-      <c r="G403">
-        <v>60.669910000000002</v>
-      </c>
-      <c r="H403">
-        <v>-170.07918000000001</v>
-      </c>
-      <c r="I403" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="K403" s="1">
-        <v>51</v>
-      </c>
-      <c r="L403" s="1">
-        <v>868</v>
-      </c>
-      <c r="M403" s="1">
-        <v>14</v>
-      </c>
-      <c r="N403" s="1">
-        <v>0</v>
-      </c>
-      <c r="O403" s="1">
-        <v>18</v>
-      </c>
-      <c r="S403" s="1">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="T403" s="1">
         <v>74.7</v>
       </c>
     </row>

</xml_diff>